<commit_message>
Adjudicate disputed rater scores in coder B sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017dFNDVoBaR63noXV5zTnsF
</commit_message>
<xml_diff>
--- a/data/human_creation_sample_filled_coderB.xlsx
+++ b/data/human_creation_sample_filled_coderB.xlsx
@@ -697,7 +697,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/1 (median used)</t>
+          <t>raters A/B/C: 0/1/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -739,11 +739,11 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -800,11 +800,11 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/2/1 (median used)</t>
+          <t>raters A/B/C: 1/2/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/1 (median used)</t>
+          <t>raters A/B/C: 0/1/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -945,11 +945,11 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1139,11 +1139,11 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1398,11 +1398,11 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/2/1 (median used)</t>
+          <t>raters A/B/C: 1/2/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/2/1 (median used)</t>
+          <t>raters A/B/C: 2/2/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/1/2 (median used)</t>
+          <t>raters A/B/C: 1/1/2; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/1 (median used)</t>
+          <t>raters A/B/C: 0/1/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/2/1 (median used)</t>
+          <t>raters A/B/C: 2/2/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/2/1 (median used)</t>
+          <t>raters A/B/C: 1/2/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/2/1 (median used)</t>
+          <t>raters A/B/C: 2/2/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/1/2 (median used)</t>
+          <t>raters A/B/C: 2/1/2; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/1/0 (median used)</t>
+          <t>raters A/B/C: 1/1/0; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/1/1 (median used)</t>
+          <t>raters A/B/C: 2/1/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/0 (median used)</t>
+          <t>raters A/B/C: 1/0/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2736,11 +2736,11 @@
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/0 (median used)</t>
+          <t>raters A/B/C: 1/0/0; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/0/2 (median used)</t>
+          <t>raters A/B/C: 2/0/2; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/1/2 (median used)</t>
+          <t>raters A/B/C: 2/1/2; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/2/1 (median used)</t>
+          <t>raters A/B/C: 1/2/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/0/2 (median used)</t>
+          <t>raters A/B/C: 2/0/2; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3027,11 +3027,11 @@
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/0/2 (median used)</t>
+          <t>raters A/B/C: 2/0/2; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3157,11 +3157,11 @@
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3245,7 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/0/2 (median used)</t>
+          <t>raters A/B/C: 2/0/2; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3375,7 +3375,7 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3569,11 +3569,11 @@
         </is>
       </c>
       <c r="D153" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/1/0 (median used)</t>
+          <t>raters A/B/C: 1/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/2/1 (median used)</t>
+          <t>raters A/B/C: 1/2/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3615,11 +3615,11 @@
         </is>
       </c>
       <c r="D155" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/2 (median used)</t>
+          <t>raters A/B/C: 1/0/2; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/1 (median used)</t>
+          <t>raters A/B/C: 0/1/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/2/1 (median used)</t>
+          <t>raters A/B/C: 1/2/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 2/0/2 (median used)</t>
+          <t>raters A/B/C: 2/0/2; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/2/0 (median used)</t>
+          <t>raters A/B/C: 0/2/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/0/1 (median used)</t>
+          <t>raters A/B/C: 1/0/1; adjudicated to 1 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 0/1/0 (median used)</t>
+          <t>raters A/B/C: 0/1/0; adjudicated to 0 per guide rules</t>
         </is>
       </c>
     </row>
@@ -4390,11 +4390,11 @@
         </is>
       </c>
       <c r="D192" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>raters A/B/C: 1/2/1 (median used)</t>
+          <t>raters A/B/C: 1/2/1; adjudicated to 2 per guide rules</t>
         </is>
       </c>
     </row>

</xml_diff>